<commit_message>
update tiến trình dự án
Thêm ControllerResult.java để chuẩn hóa dữ liệu trả về từ Controller, giữ đúng nguyên tắc MVC.

Xây dựng BaseController.java và AuthenticationState.java dạng Singleton để quản lý phiên đăng nhập an toàn toàn cục.

Giao diện an toàn (View Layer):
Sửa lỗi hỏng cấu trúc thư mục src/view & src/controller của hệ điều hành.

Phát triển tiện ích ConsoleUI.java dùng vòng lặp vô tận while-try-catch ép kiểu an toàn tuyệt đối chống crash InputMismatchException.

Code MainMenuView.java và AdminView.java. Khởi tạo Main.java làm Entry Point.

Hoàn thiện Logic Nghiệp vụ Admin:
Viết AdminController.java tích hợp logic Duyệt (approveCustomer, approveSeller).

Phân tách rõ ràng Business Logic: thêm tính năng Khóa (ban) và Mở khóa riêng biệt (unbanCustomer, unbanSeller) với điều kiện bắt lỗi khắt khe (chỉ Unban tài khoản có trạng thái BANNED).
</commit_message>
<xml_diff>
--- a/ai_logs/GiaHuy_AI_logs.xlsx
+++ b/ai_logs/GiaHuy_AI_logs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="152">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -215,6 +215,63 @@
     <t>Thiet ke lai thuat toan theo BufferedWriter Stream: sinh 1 object -&gt; ghi ngay -&gt; giai phong. RAM luon o muc ~2MB bat ke so luong dong.</t>
   </si>
   <si>
+    <t>Logic Error</t>
+  </si>
+  <si>
+    <t>AI ban đầu đề xuất viết các lệnh System.out.println("Thành công"); trực tiếp bên trong các hàm của tầng Controller để in ra màn hình cho nhanh.</t>
+  </si>
+  <si>
+    <t>Việc in dữ liệu trực tiếp từ Controller đã vi phạm nghiêm trọng nguyên tắc của mô hình MVC (Controller không được dính dáng đến UI).</t>
+  </si>
+  <si>
+    <t>Tự rà soát lại lý thuyết MVC được học trên lớp và kiểm tra chéo (Cross-check) ranh giới giữa View và Controller.</t>
+  </si>
+  <si>
+    <t>Yêu cầu AI xóa bỏ toàn bộ lệnh print. Ép AI phải thiết kế lớp ControllerResult để đóng gói dữ liệu trả về, sau đó View mới được phép lấy dữ liệu đó ra để in.</t>
+  </si>
+  <si>
+    <t>Environmental Blindness</t>
+  </si>
+  <si>
+    <t>Khi IDE báo lỗi không thể tạo class, AI ban đầu khăng khăng cho rằng lỗi là do sai cú pháp Java hoặc thiếu thư viện trong file cấu hình.</t>
+  </si>
+  <si>
+    <t>Code hoàn toàn đúng. Nguyên nhân thực tế là do hệ điều hành Windows bị lỗi, sinh ra một "file rác" 0-byte tên là controller ngăn cản việc tạo thư mục trùng tên.</t>
+  </si>
+  <si>
+    <t>Xem xét kỹ thông báo lỗi và yêu cầu AI chạy lệnh Terminal list_dir để ép nó quét trực tiếp hệ thống file vật lý thay vì chỉ đọc code.</t>
+  </si>
+  <si>
+    <t>Ra lệnh cho AI dùng PowerShell Remove-Item để xóa tận gốc file rác cấp hệ điều hành, sau đó tạo lại thư mục chuẩn.</t>
+  </si>
+  <si>
+    <t>AI đề xuất dùng hàm cơ bản scanner.nextInt() để đọc lựa chọn từ Menu của người dùng.</t>
+  </si>
+  <si>
+    <t>Trên thực tế, nếu người dùng vô tình (hoặc cố ý) nhập chữ cái "a", "b", "c" vào thì hàm nextInt() sẽ lập tức làm chương trình văng lỗi InputMismatchException và sập luôn.</t>
+  </si>
+  <si>
+    <t>Tự tay test thử chương trình (Black-box testing) bằng cách cố tình nhập sai kiểu dữ liệu tại màn hình Menu.</t>
+  </si>
+  <si>
+    <t>Phủ quyết code cũ. Yêu cầu AI xây dựng một lớp ConsoleUI.java dùng vòng lặp vô tận, đọc bằng nextLine() rồi ép kiểu bằng try-catch(NumberFormatException) để chương trình bất tử.</t>
+  </si>
+  <si>
+    <t>Business Logic Flaw</t>
+  </si>
+  <si>
+    <t>AI gộp chung tính năng: dùng một hàm approveCustomer duy nhất để duyệt tài khoản mới VÀ để mở khóa (Unban) tài khoản vi phạm.</t>
+  </si>
+  <si>
+    <t>Về mặt code thì chạy được, nhưng mất hoàn toàn tính kiểm soát (Validation). Admin có thể vô tình bấm nhầm "Mở khóa" cho một người đang hoạt động bình thường mà hệ thống không báo lỗi.</t>
+  </si>
+  <si>
+    <t>Đặt câu hỏi phản biện về Luồng người dùng (User Flow): "Nếu có Ban thì phải có Unban chuyên biệt chứ?"</t>
+  </si>
+  <si>
+    <t>Buộc AI viết hàm unbanCustomer tách biệt hoàn toàn. Thêm logic khắt khe: if (status != BANNED) throw Error. Xây dựng Unit Test để bảo vệ hàm này.</t>
+  </si>
+  <si>
     <t>HALLUCINATION TYPES REFERENCE:</t>
   </si>
   <si>
@@ -242,9 +299,6 @@
     <t>Code không handle array rỗng</t>
   </si>
   <si>
-    <t>Logic Error</t>
-  </si>
-  <si>
     <t>AI đưa kết luận sai về 'best practice'</t>
   </si>
   <si>
@@ -276,6 +330,51 @@
   </si>
   <si>
     <t>Entry # (from Sheet)</t>
+  </si>
+  <si>
+    <t>Logic Flaw</t>
+  </si>
+  <si>
+    <t>Khi được yêu cầu viết DataGenerator, AI đề xuất dùng vòng lặp for và hàm Random để chọn ngẫu nhiên Product ID bỏ vào danh sách Flash Sale.</t>
+  </si>
+  <si>
+    <t>Việc random ngẫu nhiên liên tục sẽ dẫn đến tình trạng trùng lặp Product ID trong cùng một phiên Flash Sale (Ví dụ: Sản phẩm A vừa giảm giá 10% vừa giảm 50% cùng lúc).</t>
+  </si>
+  <si>
+    <t>Chạy thử file sinh dữ liệu, mở file flash_sales.csv lên và dùng tính năng "Highlight Duplicate" của Excel thì phát hiện hàng loạt ID bị trùng.</t>
+  </si>
+  <si>
+    <t>Bắt AI phải thay đổi thuật toán: Thay vì Random trực tiếp, phải dùng Set&lt;String&gt; để lưu trữ và loại bỏ các ID trùng lặp, đảm bảo mỗi sản phẩm chỉ xuất hiện 1 lần trong đợt sale.</t>
+  </si>
+  <si>
+    <t>API Misunderstanding</t>
+  </si>
+  <si>
+    <t>AI khẳng định rằng chỉ cần thêm từ khóa synchronized vào hàm placeOrder() là đủ để chống Race Condition khi có 1000 người mua hàng cùng lúc.</t>
+  </si>
+  <si>
+    <t>synchronized chỉ có tác dụng khóa luồng (Thread) bên trong cùng một máy ảo JVM. Vì database của chúng ta là file CSV, nếu chạy 2 cửa sổ Terminal (2 JVM) cùng mua hàng, file CSV vẫn bị ghi đè và rách dữ liệu.</t>
+  </si>
+  <si>
+    <t>Chạy Simulator nghiệm thu: Mở 2 cửa sổ Terminal chạy độc lập cùng mua 1 món hàng. Kết quả số lượng tồn kho vẫn bị âm (Negative Inventory).</t>
+  </si>
+  <si>
+    <t>Phủ quyết AI. Yêu cầu AI nghiên cứu thư viện java.nio và sử dụng FileChannel.lock() để thực hiện OS-level Lock (Khóa ở cấp hệ điều hành) thay vì khóa cấp JVM.</t>
+  </si>
+  <si>
+    <t>Architectural Violation</t>
+  </si>
+  <si>
+    <t>AI gợi ý lưu thông tin người dùng đang đăng nhập vào một biến public static Customer currentUser đặt ngay bên trong class Entity Customer cho dễ gọi.</t>
+  </si>
+  <si>
+    <t>Việc lưu trạng thái phiên làm việc (Session State) vào trong một class Entity là vi phạm nghiêm trọng nguyên lý Single Responsibility (SRP) của OOP. Entity chỉ dùng để chứa cấu trúc dữ liệu.</t>
+  </si>
+  <si>
+    <t>Review lại code theo chuẩn MVC của giảng viên. Nhận thấy nếu sau này app nâng cấp lên Web, biến static sẽ làm toàn bộ người dùng dùng chung 1 tài khoản.</t>
+  </si>
+  <si>
+    <t>Bắt AI xóa bỏ biến static trong Model. Yêu cầu thiết kế một lớp AuthenticationState dạng Singleton nằm ở tầng Controller để quản lý phiên đăng nhập độc lập.</t>
   </si>
   <si>
     <t>SELF-ASSESSMENT CHECKLIST (Trước khi nộp)</t>
@@ -400,7 +499,7 @@
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -487,14 +586,6 @@
       <i/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -520,13 +611,6 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1024,19 +1108,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1045,131 +1138,122 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1206,23 +1290,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1244,7 +1342,7 @@
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1579,14 +1677,14 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="21" spans="1:6">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" s="1" customFormat="1" ht="18.75" spans="1:1">
       <c r="A3" s="4" t="s">
@@ -1594,7 +1692,7 @@
       </c>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:3">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="30" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1602,7 +1700,7 @@
       </c>
     </row>
     <row r="5" s="1" customFormat="1" spans="1:3">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="30" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1610,7 +1708,7 @@
       </c>
     </row>
     <row r="6" s="1" customFormat="1" spans="1:3">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="30" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -1618,7 +1716,7 @@
       </c>
     </row>
     <row r="7" s="1" customFormat="1" spans="1:3">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="30" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1631,35 +1729,35 @@
       </c>
     </row>
     <row r="10" s="1" customFormat="1" spans="1:3">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="31" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="1" spans="1:3">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="32">
         <v>18</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="1" spans="1:5">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="33">
         <v>0.16</v>
       </c>
-      <c r="E12" s="30"/>
+      <c r="E12" s="34"/>
     </row>
     <row r="13" s="1" customFormat="1" spans="1:3">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="32">
         <v>2</v>
       </c>
     </row>
@@ -1758,7 +1856,7 @@
       <c r="A24" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="31">
+      <c r="B24" s="35">
         <v>2</v>
       </c>
       <c r="C24" s="14" t="s">
@@ -1769,7 +1867,7 @@
       <c r="A25" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="35">
         <v>2</v>
       </c>
       <c r="C25" s="14" t="s">
@@ -1780,7 +1878,7 @@
       <c r="A26" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="31">
+      <c r="B26" s="35">
         <v>2</v>
       </c>
       <c r="C26" s="14" t="s">
@@ -1791,7 +1889,7 @@
       <c r="A27" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="31">
+      <c r="B27" s="35">
         <v>2</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -1820,12 +1918,12 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="21" spans="1:1">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="25" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="26" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1850,79 +1948,129 @@
       </c>
     </row>
     <row r="4" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A4" s="23">
+      <c r="A4" s="27">
+        <v>1</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" ht="75" spans="1:6">
+      <c r="A5" s="27">
+        <v>2</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
+      <c r="A6" s="27">
+        <v>3</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
+      <c r="A7" s="27">
+        <v>4</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
+      <c r="A8" s="27">
         <v>5</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B8" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="75" spans="1:6">
-      <c r="A5" s="23">
-        <v>4</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-    </row>
-    <row r="8" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
+      <c r="C8" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="9" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
+      <c r="A9" s="27">
+        <v>6</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="10" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A10" s="15"/>
+      <c r="A10" s="27">
+        <v>7</v>
+      </c>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
@@ -1930,7 +2078,9 @@
       <c r="F10" s="15"/>
     </row>
     <row r="11" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A11" s="15"/>
+      <c r="A11" s="27">
+        <v>8</v>
+      </c>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -1938,7 +2088,9 @@
       <c r="F11" s="15"/>
     </row>
     <row r="12" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A12" s="15"/>
+      <c r="A12" s="27">
+        <v>9</v>
+      </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
       <c r="D12" s="15"/>
@@ -1946,7 +2098,9 @@
       <c r="F12" s="15"/>
     </row>
     <row r="13" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A13" s="15"/>
+      <c r="A13" s="27">
+        <v>10</v>
+      </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
@@ -1954,7 +2108,9 @@
       <c r="F13" s="15"/>
     </row>
     <row r="14" s="1" customFormat="1" ht="60" customHeight="1" spans="1:6">
-      <c r="A14" s="15"/>
+      <c r="A14" s="27">
+        <v>11</v>
+      </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -2043,29 +2199,29 @@
     </row>
     <row r="30" s="1" customFormat="1" ht="18.75" spans="1:1">
       <c r="A30" s="4" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" s="1" customFormat="1" spans="1:3">
       <c r="A31" s="13" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" s="1" customFormat="1" ht="30" spans="1:3">
       <c r="A32" s="15" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" s="1" customFormat="1" ht="30" spans="1:3">
@@ -2073,43 +2229,43 @@
         <v>52</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" s="1" customFormat="1" ht="30" spans="1:3">
       <c r="A34" s="15" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" ht="30" spans="1:3">
       <c r="A35" s="15" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" s="1" customFormat="1" ht="45" spans="1:3">
       <c r="A36" s="15" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2125,90 +2281,326 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="5"/>
+  <dimension ref="A1:F43"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="12.6285714285714" customWidth="1"/>
-    <col min="2" max="2" width="18.6285714285714" customWidth="1"/>
-    <col min="3" max="3" width="30.6285714285714" customWidth="1"/>
-    <col min="4" max="4" width="35.6285714285714" customWidth="1"/>
-    <col min="5" max="5" width="30.6285714285714" customWidth="1"/>
-    <col min="6" max="6" width="35.6285714285714" customWidth="1"/>
+    <col min="1" max="1" width="12.6285714285714" style="16" customWidth="1"/>
+    <col min="2" max="2" width="18.6285714285714" style="16" customWidth="1"/>
+    <col min="3" max="3" width="30.6285714285714" style="16" customWidth="1"/>
+    <col min="4" max="4" width="35.6285714285714" style="16" customWidth="1"/>
+    <col min="5" max="5" width="30.6285714285714" style="16" customWidth="1"/>
+    <col min="6" max="6" width="35.6285714285714" style="16" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:6">
-      <c r="A1" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="A1" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="18" t="s">
-        <v>80</v>
+      <c r="A2" s="19" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="3" ht="30" spans="1:6">
-      <c r="A3" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="19" t="s">
+      <c r="A3" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4" ht="80.1" customHeight="1" spans="1:6">
-      <c r="A4" s="20">
+      <c r="A4" s="21">
+        <v>1</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" ht="80.1" customHeight="1" spans="1:6">
+      <c r="A5" s="21">
+        <v>2</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1" spans="1:6">
+      <c r="A6" s="21">
+        <v>3</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1" spans="1:6">
+      <c r="A7" s="21">
+        <v>4</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1" spans="1:6">
+      <c r="A8" s="21">
         <v>5</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" ht="80.1" customHeight="1" spans="1:6">
-      <c r="A5" s="20">
-        <v>4</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>60</v>
+      <c r="B8" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" spans="1:1">
+      <c r="A9" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1" spans="1:1">
+      <c r="A10" s="21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1" spans="1:1">
+      <c r="A11" s="21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1" spans="1:1">
+      <c r="A12" s="21">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1" spans="1:1">
+      <c r="A13" s="21">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1" spans="1:1">
+      <c r="A14" s="21">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1" spans="1:1">
+      <c r="A15" s="21">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" spans="1:1">
+      <c r="A16" s="21">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1" spans="1:1">
+      <c r="A17" s="21">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1" spans="1:1">
+      <c r="A18" s="21">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1" spans="1:1">
+      <c r="A19" s="21">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1" spans="1:1">
+      <c r="A20" s="21">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1" spans="1:1">
+      <c r="A21" s="21">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1" spans="1:1">
+      <c r="A22" s="21">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1" spans="1:1">
+      <c r="A23" s="21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1" spans="1:1">
+      <c r="A24" s="21">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1" spans="1:1">
+      <c r="A25" s="21">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1" spans="1:1">
+      <c r="A26" s="21">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1" spans="1:1">
+      <c r="A27" s="21">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1" spans="1:1">
+      <c r="A28" s="21">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1" spans="1:1">
+      <c r="A29" s="21">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1" spans="1:1">
+      <c r="A30" s="21">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1" spans="1:1">
+      <c r="A31" s="21">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1" spans="1:1">
+      <c r="A32" s="21">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1" spans="1:1">
+      <c r="A33" s="21">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1" spans="1:1">
+      <c r="A34" s="21">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1" spans="1:1">
+      <c r="A35" s="21">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" ht="90" customHeight="1" spans="1:1">
+      <c r="A36" s="21">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" ht="90" customHeight="1" spans="1:1">
+      <c r="A37" s="21">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" ht="90" customHeight="1" spans="1:1">
+      <c r="A38" s="21">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" ht="90" customHeight="1" spans="1:1">
+      <c r="A39" s="21">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" ht="90" customHeight="1" spans="1:1">
+      <c r="A40" s="21">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" ht="90" customHeight="1" spans="1:1">
+      <c r="A41" s="21">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" ht="90" customHeight="1" spans="1:1">
+      <c r="A42" s="21">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" ht="90" customHeight="1" spans="1:1">
+      <c r="A43" s="21">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -2236,42 +2628,42 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="21" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:1">
       <c r="A2" s="3" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" ht="18.75" spans="1:1">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" spans="1:4">
       <c r="A5" s="5" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" spans="1:4">
       <c r="A6" s="7" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>34</v>
@@ -2279,13 +2671,13 @@
     </row>
     <row r="7" s="1" customFormat="1" spans="1:4">
       <c r="A7" s="7" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>34</v>
@@ -2293,13 +2685,13 @@
     </row>
     <row r="8" s="1" customFormat="1" spans="1:4">
       <c r="A8" s="7" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>34</v>
@@ -2307,13 +2699,13 @@
     </row>
     <row r="9" s="1" customFormat="1" spans="1:4">
       <c r="A9" s="7" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>34</v>
@@ -2321,13 +2713,13 @@
     </row>
     <row r="10" s="1" customFormat="1" spans="1:4">
       <c r="A10" s="7" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>34</v>
@@ -2335,32 +2727,32 @@
     </row>
     <row r="12" s="1" customFormat="1" ht="18.75" spans="1:1">
       <c r="A12" s="4" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="1" spans="1:4">
       <c r="A13" s="5" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" spans="1:4">
       <c r="A14" s="7" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>34</v>
@@ -2368,13 +2760,13 @@
     </row>
     <row r="15" s="1" customFormat="1" spans="1:4">
       <c r="A15" s="7" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>34</v>
@@ -2382,13 +2774,13 @@
     </row>
     <row r="16" s="1" customFormat="1" spans="1:4">
       <c r="A16" s="7" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>34</v>
@@ -2396,13 +2788,13 @@
     </row>
     <row r="17" s="1" customFormat="1" spans="1:4">
       <c r="A17" s="7" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>34</v>
@@ -2410,13 +2802,13 @@
     </row>
     <row r="18" s="1" customFormat="1" spans="1:4">
       <c r="A18" s="7" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>34</v>
@@ -2424,46 +2816,46 @@
     </row>
     <row r="20" s="1" customFormat="1" ht="15.75" spans="1:1">
       <c r="A20" s="9" t="s">
-        <v>107</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" spans="1:1">
       <c r="A21" s="10" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" s="1" customFormat="1" spans="1:1">
       <c r="A22" s="10" t="s">
-        <v>109</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" s="1" customFormat="1" ht="18.75" spans="1:1">
       <c r="A25" s="4" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" s="1" customFormat="1" spans="1:1">
       <c r="A26" s="11" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" s="1" customFormat="1" ht="45" spans="1:4">
       <c r="A27" s="12" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" spans="1:4">
       <c r="A28" s="14" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>34</v>
@@ -2477,7 +2869,7 @@
     </row>
     <row r="29" s="1" customFormat="1" spans="1:4">
       <c r="A29" s="14" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>34</v>
@@ -2491,7 +2883,7 @@
     </row>
     <row r="30" s="1" customFormat="1" spans="1:4">
       <c r="A30" s="14" t="s">
-        <v>118</v>
+        <v>151</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>34</v>

</xml_diff>